<commit_message>
Beautified mark attendance page and fixed login
</commit_message>
<xml_diff>
--- a/attendance_log.xlsx
+++ b/attendance_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,6 +536,54 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Vinod Karri</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2025-06-13 08:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Vinod Karri</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2025-06-13 08:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Vinod Karri</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2025-06-13 08:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Vinod Karri</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2025-06-13 09:01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>